<commit_message>
feat: modal nativo para exportacao csv e consistencia visual das janelas de confirmacao
- Integramos interop entre JS e C# com `window.external.sendMessage` e `RegisterWebMessageReceivedHandler` no Photino.
- Agora, a exportacao de CSV exibe a janela nativa do OS `ShowSaveFile` com memoria do diretorio mais recente.
- Substituidos todos os modais de `alert` e `confirm` remanescentes de componentes filhos pelo `confirmDialog` robusto da aplicacao para garantir experiencia 100% Desktop-Native.
</commit_message>
<xml_diff>
--- a/CONTROLE PAGAMENTOS.xlsx
+++ b/CONTROLE PAGAMENTOS.xlsx
@@ -1954,7 +1954,7 @@
         <v>10000</v>
       </c>
       <c r="F2" s="9">
-        <v>45894</v>
+        <v>46303</v>
       </c>
       <c r="G2" s="9">
         <v>45894</v>
@@ -1976,15 +1976,15 @@
       </c>
       <c r="L2" t="str" s="12">
         <f>IF(OR(ISBLANK(PARCELAS[[#This Row],[DATA PAGAMENTO]]),DAY(PARCELAS[[#This Row],[DATA PAGAMENTO]])=0),"",TEXT(DAY(PARCELAS[[#This Row],[DATA PAGAMENTO]]),"00"))</f>
-        <v>25</v>
+        <v>08</v>
       </c>
       <c r="M2" t="str" s="13">
         <f>IF(ISBLANK(PARCELAS[[#This Row],[DATA PAGAMENTO]]),"",INDEX(MESES[MÊS],MATCH(MONTH(PARCELAS[[#This Row],[DATA PAGAMENTO]]),MESES[N],0)))</f>
-        <v>agosto</v>
+        <v>outubro</v>
       </c>
       <c r="N2" s="12">
         <f>IF(OR(ISBLANK(PARCELAS[[#This Row],[DATA PAGAMENTO]]),YEAR(PARCELAS[[#This Row],[DATA PAGAMENTO]])=1900),"",YEAR(PARCELAS[[#This Row],[DATA PAGAMENTO]]))</f>
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="O2" t="s">
         <v>43</v>

</xml_diff>